<commit_message>
Apply review fixes to the history ledger
Add FY2016 and FY2022 cash from operations from release comparatives,
carry the unchanged regular dividend across four unsourced years as
derived, and set two acquisition counts that covered only disclosed
major deals to gap.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FMM8EPvNnZesHZkQW6435U
</commit_message>
<xml_diff>
--- a/analysis/constellation-software/history-2007-2025/history_metrics.xlsx
+++ b/analysis/constellation-software/history-2007-2025/history_metrics.xlsx
@@ -648,6 +648,9 @@
       <c r="L7" t="n">
         <v>8.119999999999999</v>
       </c>
+      <c r="M7" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -808,21 +811,39 @@
       <c r="D11" t="n">
         <v>9.73</v>
       </c>
+      <c r="E11" t="n">
+        <v>23.1</v>
+      </c>
       <c r="F11" t="n">
         <v>18.59</v>
       </c>
+      <c r="G11" t="n">
+        <v>2.37</v>
+      </c>
+      <c r="H11" t="n">
+        <v>36.27</v>
+      </c>
       <c r="I11" t="n">
         <v>45.09</v>
       </c>
       <c r="J11" t="n">
         <v>100.29</v>
       </c>
+      <c r="K11" t="n">
+        <v>23.17</v>
+      </c>
       <c r="L11" t="n">
         <v>18.64</v>
       </c>
+      <c r="M11" t="n">
+        <v>4</v>
+      </c>
       <c r="N11" t="n">
         <v>216.9</v>
       </c>
+      <c r="O11" t="n">
+        <v>132.14</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -857,6 +878,9 @@
       <c r="L12" t="n">
         <v>21.85</v>
       </c>
+      <c r="M12" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1035,9 +1059,15 @@
       <c r="L16" t="n">
         <v>41.67</v>
       </c>
+      <c r="M16" t="n">
+        <v>4</v>
+      </c>
       <c r="N16" t="n">
         <v>-454</v>
       </c>
+      <c r="O16" t="n">
+        <v>-538.76</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1051,14 +1081,26 @@
       <c r="D17" t="n">
         <v>7.73</v>
       </c>
+      <c r="E17" t="n">
+        <v>19.59</v>
+      </c>
       <c r="F17" t="n">
         <v>12.88</v>
       </c>
+      <c r="G17" t="n">
+        <v>2.53</v>
+      </c>
+      <c r="H17" t="n">
+        <v>123.36</v>
+      </c>
       <c r="I17" t="n">
         <v>187.57</v>
       </c>
       <c r="J17" t="n">
         <v>312.51</v>
+      </c>
+      <c r="K17" t="n">
+        <v>61.21</v>
       </c>
       <c r="L17" t="n">
         <v>40.25</v>
@@ -1222,7 +1264,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1610,6 +1652,60 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>acquisition_count</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>FY2015</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>[3]</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>['https://tracxn.com/d/acquisitions/acquisitions-by-constellation-software/__YaRluimuGqgVfqr0Xhgb2dPWiMKnmgzXPcPNPni5Ssg']</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Set to gap by Fable review 2026-09-14: the figure counts publicly announced major deals, not the company's total for FY2015; Constellation closes dozens of small acquisitions a year, so 3 is not a total.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>acquisition_count</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>FY2019</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>[3]</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>['https://nicoper.substack.com/p/4-constellation-acquisitions-2022']</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Set to gap by Fable review 2026-09-14: the figure counts publicly announced major deals, not the company's total for FY2019; Constellation closes dozens of small acquisitions a year, so 3 is not a total.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1621,7 +1717,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G192"/>
+  <dimension ref="A1:G198"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5496,16 +5592,16 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>fcfa2s</t>
+          <t>cash_from_operations</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>FY2018</t>
+          <t>FY2016</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>559</v>
+        <v>491</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
@@ -5519,28 +5615,28 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2020/02/13/1984977/0/en/Constellation-Software-Inc-Announces-Results-for-the-Fourth-Quarter-and-Year-Ended-December-31-2019-and-Declares-Quarterly-Dividend.html</t>
+          <t>https://www.globenewswire.com/news-release/2018/02/14/1348408/0/en/Constellation-Software-Inc-Announces-Results-for-the-Fourth-Quarter-and-Year-Ended-December-31-2017-and-Declares-Quarterly-Dividend.html</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>Reused from long-term-hold/holdings.json parent_long_run.</t>
+          <t>Comparative figure stated in the FY2017 annual release ('increase of 8%/$37M over $491M in 2016'). Added by Fable review 2026-09-14.</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>fcfa2s</t>
+          <t>cash_from_operations</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>FY2019</t>
+          <t>FY2022</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>590</v>
+        <v>1297</v>
       </c>
       <c r="D116" t="inlineStr">
         <is>
@@ -5554,12 +5650,12 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2020/02/13/1984977/0/en/Constellation-Software-Inc-Announces-Results-for-the-Fourth-Quarter-and-Year-Ended-December-31-2019-and-Declares-Quarterly-Dividend.html</t>
+          <t>https://www.globenewswire.com/news-release/2023/03/29/2637195/0/en/Constellation-Software-Inc-Announces-Results-for-the-Fourth-Quarter-and-Year-Ended-December-31-2022-and-Declares-Quarterly-Dividend.html</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>Reused from parent_long_run. 6% increase over FY2018.</t>
+          <t>Release states CFO of $1,297 million for 2022, a decrease of $2 million from $1,300 million in 2021. Added by Fable review 2026-09-14 from a WebSearch snippet.</t>
         </is>
       </c>
     </row>
@@ -5571,11 +5667,11 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>FY2020</t>
+          <t>FY2018</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>989</v>
+        <v>559</v>
       </c>
       <c r="D117" t="inlineStr">
         <is>
@@ -5589,12 +5685,12 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2021/02/12/2175170/0/en/Constellation-Software-Inc-Announces-Results-for-the-Fourth-Quarter-and-Year-Ended-December-31-2020-and-Declares-Quarterly-Dividend.html</t>
+          <t>https://www.globenewswire.com/news-release/2020/02/13/1984977/0/en/Constellation-Software-Inc-Announces-Results-for-the-Fourth-Quarter-and-Year-Ended-December-31-2019-and-Declares-Quarterly-Dividend.html</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>Reused from parent_long_run. +68%/$399M over FY2019.</t>
+          <t>Reused from long-term-hold/holdings.json parent_long_run.</t>
         </is>
       </c>
     </row>
@@ -5606,11 +5702,11 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>FY2021</t>
+          <t>FY2019</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>883</v>
+        <v>590</v>
       </c>
       <c r="D118" t="inlineStr">
         <is>
@@ -5624,12 +5720,12 @@
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2022/02/10/2383319/0/en/Constellation-Software-Inc-Announces-Results-for-the-Fourth-Quarter-and-Year-Ended-December-31-2021-and-Declares-Quarterly-Dividend.html</t>
+          <t>https://www.globenewswire.com/news-release/2020/02/13/1984977/0/en/Constellation-Software-Inc-Announces-Results-for-the-Fourth-Quarter-and-Year-Ended-December-31-2019-and-Declares-Quarterly-Dividend.html</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>Reused from parent_long_run. -11%/$106M vs FY2020, mainly the TSS/IRGA revaluation charge and Topicus.com non-controlling interests.</t>
+          <t>Reused from parent_long_run. 6% increase over FY2018.</t>
         </is>
       </c>
     </row>
@@ -5641,11 +5737,11 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>FY2022</t>
+          <t>FY2020</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>853</v>
+        <v>989</v>
       </c>
       <c r="D119" t="inlineStr">
         <is>
@@ -5659,12 +5755,12 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>https://www.csisoftware.com/docs/default-source/investor-relations/statutory-filings/csi---mda-q4-2023---final.pdf?sfvrsn=47d7de81_3</t>
+          <t>https://www.globenewswire.com/news-release/2021/02/12/2175170/0/en/Constellation-Software-Inc-Announces-Results-for-the-Fourth-Quarter-and-Year-Ended-December-31-2020-and-Declares-Quarterly-Dividend.html</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>Reused from ledger.json.</t>
+          <t>Reused from parent_long_run. +68%/$399M over FY2019.</t>
         </is>
       </c>
     </row>
@@ -5676,11 +5772,11 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>FY2023</t>
+          <t>FY2021</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>1160</v>
+        <v>883</v>
       </c>
       <c r="D120" t="inlineStr">
         <is>
@@ -5694,12 +5790,12 @@
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2024/03/06/2841834/0/en/Constellation-Software-Inc-Announces-Results-for-the-Fourth-Quarter-and-Year-Ended-December-31-2023-and-Declares-Quarterly-Dividend.html</t>
+          <t>https://www.globenewswire.com/news-release/2022/02/10/2383319/0/en/Constellation-Software-Inc-Announces-Results-for-the-Fourth-Quarter-and-Year-Ended-December-31-2021-and-Declares-Quarterly-Dividend.html</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>Reused from ledger.json.</t>
+          <t>Reused from parent_long_run. -11%/$106M vs FY2020, mainly the TSS/IRGA revaluation charge and Topicus.com non-controlling interests.</t>
         </is>
       </c>
     </row>
@@ -5711,11 +5807,11 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>FY2024</t>
+          <t>FY2022</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>1472</v>
+        <v>853</v>
       </c>
       <c r="D121" t="inlineStr">
         <is>
@@ -5729,7 +5825,7 @@
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>https://www.csisoftware.com/constellation-software-inc-announces-results-for-the-fourth-quarter-and-year-ended-december-31-2024-and-declares-quarterly-dividend/</t>
+          <t>https://www.csisoftware.com/docs/default-source/investor-relations/statutory-filings/csi---mda-q4-2023---final.pdf?sfvrsn=47d7de81_3</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
@@ -5746,11 +5842,11 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>FY2025</t>
+          <t>FY2023</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>1683</v>
+        <v>1160</v>
       </c>
       <c r="D122" t="inlineStr">
         <is>
@@ -5764,32 +5860,32 @@
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2026/03/09/3251696/0/en/constellation-software-inc-announces-results-for-the-fourth-quarter-and-year-ended-december-31-2025-and-declares-quarterly-dividend.html</t>
+          <t>https://www.globenewswire.com/news-release/2024/03/06/2841834/0/en/Constellation-Software-Inc-Announces-Results-for-the-Fourth-Quarter-and-Year-Ended-December-31-2023-and-Declares-Quarterly-Dividend.html</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>Reused from ledger.json. +$210M/14% over FY2024's $1,472M.</t>
+          <t>Reused from ledger.json.</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>acquisitions_cash_spent</t>
+          <t>fcfa2s</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>FY2008</t>
+          <t>FY2024</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>94</v>
+        <v>1472</v>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>USD millions approximate</t>
+          <t>USD millions</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -5799,28 +5895,28 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>https://www.mbi-deepdives.com/content/files/2022/07/Constellation-Software-SH-Letters-Merged.pdf</t>
+          <t>https://www.csisoftware.com/constellation-software-inc-announces-results-for-the-fourth-quarter-and-year-ended-december-31-2024-and-declares-quarterly-dividend/</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>2008 President's letter: ~$94M of capital deployed/committed in 2008 (Maximus assets, 16 other businesses, VMS share purchases, pending Gladstone plc offer). This is total capital deployed/committed, not strictly cash spent on closed acquisitions.</t>
+          <t>Reused from ledger.json.</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>acquisitions_cash_spent</t>
+          <t>fcfa2s</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>FY2013</t>
+          <t>FY2025</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>558</v>
+        <v>1683</v>
       </c>
       <c r="D124" t="inlineStr">
         <is>
@@ -5834,12 +5930,12 @@
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1113678/000119312514275886/d757774dex21.htm</t>
+          <t>https://www.globenewswire.com/news-release/2026/03/09/3251696/0/en/constellation-software-inc-announces-results-for-the-fourth-quarter-and-year-ended-december-31-2025-and-declares-quarterly-dividend.html</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>Thirty acquisitions for aggregate cash consideration of $558M (plus $27M holdbacks and $4M contingent consideration, not included). Includes the TSS acquisition, closed Dec 31, 2013.</t>
+          <t>Reused from ledger.json. +$210M/14% over FY2024's $1,472M.</t>
         </is>
       </c>
     </row>
@@ -5851,15 +5947,15 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>FY2014</t>
+          <t>FY2008</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>115</v>
+        <v>94</v>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>USD millions</t>
+          <t>USD millions approximate</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
@@ -5869,12 +5965,12 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1113678/000119312515138334/d906182dex26.htm</t>
+          <t>https://www.mbi-deepdives.com/content/files/2022/07/Constellation-Software-SH-Letters-Merged.pdf</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>23 acquisitions for aggregate cash consideration of $115M (plus $17M holdbacks, $8M contingent consideration, not included).</t>
+          <t>2008 President's letter: ~$94M of capital deployed/committed in 2008 (Maximus assets, 16 other businesses, VMS share purchases, pending Gladstone plc offer). This is total capital deployed/committed, not strictly cash spent on closed acquisitions.</t>
         </is>
       </c>
     </row>
@@ -5886,11 +5982,11 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>FY2015</t>
+          <t>FY2013</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>248.8</v>
+        <v>558</v>
       </c>
       <c r="D126" t="inlineStr">
         <is>
@@ -5904,12 +6000,12 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>https://www.csisoftware.com/docs/default-source/investor-relations/statutory-filings/sr_q4_2015.pdf</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1113678/000119312514275886/d757774dex21.htm</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>Aggregate of $248.8M, including holdback payments on prior acquisitions -- not directly comparable line-for-line with the FY2013/FY2014 figures above.</t>
+          <t>Thirty acquisitions for aggregate cash consideration of $558M (plus $27M holdbacks and $4M contingent consideration, not included). Includes the TSS acquisition, closed Dec 31, 2013.</t>
         </is>
       </c>
     </row>
@@ -5921,11 +6017,11 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>FY2016</t>
+          <t>FY2014</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>178.1</v>
+        <v>115</v>
       </c>
       <c r="D127" t="inlineStr">
         <is>
@@ -5939,12 +6035,12 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>https://www.csisoftware.com/docs/default-source/investor-relations/statutory-filings/mda_q4_2016.pdf</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1113678/000119312515138334/d906182dex26.htm</t>
         </is>
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>Reused from long-term-hold/holdings.json parent_long_run (mda_q4_2016.pdf). This project's own FY2012-2016 intake sweep did not locate this figure and recorded it as a gap; parent_long_run already held it.</t>
+          <t>23 acquisitions for aggregate cash consideration of $115M (plus $17M holdbacks, $8M contingent consideration, not included).</t>
         </is>
       </c>
     </row>
@@ -5956,11 +6052,11 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>FY2018</t>
+          <t>FY2015</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>603</v>
+        <v>248.8</v>
       </c>
       <c r="D128" t="inlineStr">
         <is>
@@ -5974,10 +6070,14 @@
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2019/02/14/1725078/0/en/Constellation-Software-Inc-Announces-Results-for-the-Fourth-Quarter-and-Year-Ended-December-31-2018-and-Declares-Quarterly-and-Special-Dividends.html</t>
-        </is>
-      </c>
-      <c r="G128" t="inlineStr"/>
+          <t>https://www.csisoftware.com/docs/default-source/investor-relations/statutory-filings/sr_q4_2015.pdf</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>Aggregate of $248.8M, including holdback payments on prior acquisitions -- not directly comparable line-for-line with the FY2013/FY2014 figures above.</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -5987,15 +6087,15 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>FY2019</t>
+          <t>FY2016</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>688</v>
+        <v>178.1</v>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>USD millions, total consideration</t>
+          <t>USD millions</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
@@ -6005,12 +6105,12 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2020/02/13/1984977/0/en/Constellation-Software-Inc-Announces-Results-for-the-Fourth-Quarter-and-Year-Ended-December-31-2019-and-Declares-Quarterly-Dividend.html</t>
+          <t>https://www.csisoftware.com/docs/default-source/investor-relations/statutory-filings/mda_q4_2016.pdf</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>'Completed acquisitions totaling $688 million in consideration during 2019', directly quoted from the FY2019 release. A $549M 'aggregate cash consideration including acquired cash' figure sourced to the 2019 AIF (confidence third_party in this project's intake, and used in parent_long_run) is recorded as a conflict; the company-quoted $688M total-consideration figure is preferred.</t>
+          <t>Reused from long-term-hold/holdings.json parent_long_run (mda_q4_2016.pdf). This project's own FY2012-2016 intake sweep did not locate this figure and recorded it as a gap; parent_long_run already held it.</t>
         </is>
       </c>
     </row>
@@ -6022,32 +6122,28 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>FY2020</t>
+          <t>FY2018</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>179</v>
+        <v>603</v>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>USD millions, aggregate cash consideration including acquired cash</t>
+          <t>USD millions</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>third_party</t>
+          <t>company</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2021/02/12/2175170/0/en/Constellation-Software-Inc-Announces-Results-for-the-Fourth-Quarter-and-Year-Ended-December-31-2020-and-Declares-Quarterly-Dividend.html</t>
-        </is>
-      </c>
-      <c r="G130" t="inlineStr">
-        <is>
-          <t>WebSearch summary attributed this to FY2020 disclosures but did not quote it directly from the release text; no company-confirmed figure was found for FY2020. Matches parent_long_run and ledger.json.</t>
-        </is>
-      </c>
+          <t>https://www.globenewswire.com/news-release/2019/02/14/1725078/0/en/Constellation-Software-Inc-Announces-Results-for-the-Fourth-Quarter-and-Year-Ended-December-31-2018-and-Declares-Quarterly-and-Special-Dividends.html</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -6057,15 +6153,15 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>FY2021</t>
+          <t>FY2019</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>1337</v>
+        <v>688</v>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>USD millions, aggregate including holdback payments, net of a $33M additional subscription related to Topicus.com B.V.</t>
+          <t>USD millions, total consideration</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
@@ -6075,12 +6171,12 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>https://www.csisoftware.com/docs/default-source/press-releases/csi---mda-q4-2021---final.pdf</t>
+          <t>https://www.globenewswire.com/news-release/2020/02/13/1984977/0/en/Constellation-Software-Inc-Announces-Results-for-the-Fourth-Quarter-and-Year-Ended-December-31-2019-and-Declares-Quarterly-Dividend.html</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>Reused from parent_long_run (Q4 2021 MD&amp;A). A separate company-sourced $1,517M 'total consideration including holdbacks, contingent consideration and amounts related to Topicus.com B.V.' figure was found independently in this project's own FY2021 release search and is recorded as a conflict (net vs. total consideration are different bases).</t>
+          <t>'Completed acquisitions totaling $688 million in consideration during 2019', directly quoted from the FY2019 release. A $549M 'aggregate cash consideration including acquired cash' figure sourced to the 2019 AIF (confidence third_party in this project's intake, and used in parent_long_run) is recorded as a conflict; the company-quoted $688M total-consideration figure is preferred.</t>
         </is>
       </c>
     </row>
@@ -6092,15 +6188,15 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>FY2022</t>
+          <t>FY2020</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>1600</v>
+        <v>179</v>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>USD millions</t>
+          <t>USD millions, aggregate cash consideration including acquired cash</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
@@ -6110,12 +6206,12 @@
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>https://www.speedwellmemos.com/p/constellation-software-2022-earnings</t>
+          <t>https://www.globenewswire.com/news-release/2021/02/12/2175170/0/en/Constellation-Software-Inc-Announces-Results-for-the-Fourth-Quarter-and-Year-Ended-December-31-2020-and-Declares-Quarterly-Dividend.html</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>No company-disclosed aggregate acquisition spend was found for FY2022; matches ledger.json and parent_long_run, all citing the same third-party source.</t>
+          <t>WebSearch summary attributed this to FY2020 disclosures but did not quote it directly from the release text; no company-confirmed figure was found for FY2020. Matches parent_long_run and ledger.json.</t>
         </is>
       </c>
     </row>
@@ -6127,15 +6223,15 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>FY2023</t>
+          <t>FY2021</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>732</v>
+        <v>1337</v>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>USD millions</t>
+          <t>USD millions, aggregate including holdback payments, net of a $33M additional subscription related to Topicus.com B.V.</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
@@ -6145,10 +6241,14 @@
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2024/03/06/2841834/0/en/Constellation-Software-Inc-Announces-Results-for-the-Fourth-Quarter-and-Year-Ended-December-31-2023-and-Declares-Quarterly-Dividend.html</t>
-        </is>
-      </c>
-      <c r="G133" t="inlineStr"/>
+          <t>https://www.csisoftware.com/docs/default-source/press-releases/csi---mda-q4-2021---final.pdf</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>Reused from parent_long_run (Q4 2021 MD&amp;A). A separate company-sourced $1,517M 'total consideration including holdbacks, contingent consideration and amounts related to Topicus.com B.V.' figure was found independently in this project's own FY2021 release search and is recorded as a conflict (net vs. total consideration are different bases).</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -6158,11 +6258,11 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>FY2024</t>
+          <t>FY2022</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>1792</v>
+        <v>1600</v>
       </c>
       <c r="D134" t="inlineStr">
         <is>
@@ -6171,15 +6271,19 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>company</t>
+          <t>third_party</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2025/03/07/3039269/0/en/Constellation-Software-Inc-Announces-Results-for-the-Fourth-Quarter-and-Year-Ended-December-31-2024-and-Declares-Quarterly-Dividend.html</t>
-        </is>
-      </c>
-      <c r="G134" t="inlineStr"/>
+          <t>https://www.speedwellmemos.com/p/constellation-software-2022-earnings</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>No company-disclosed aggregate acquisition spend was found for FY2022; matches ledger.json and parent_long_run, all citing the same third-party source.</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -6189,11 +6293,11 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>FY2025</t>
+          <t>FY2023</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>1579</v>
+        <v>732</v>
       </c>
       <c r="D135" t="inlineStr">
         <is>
@@ -6207,32 +6311,28 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2026/03/09/3251696/0/en/constellation-software-inc-announces-results-for-the-fourth-quarter-and-year-ended-december-31-2025-and-declares-quarterly-dividend.html</t>
-        </is>
-      </c>
-      <c r="G135" t="inlineStr">
-        <is>
-          <t>Total acquisition consideration of $1,579M including holdbacks and contingent consideration.</t>
-        </is>
-      </c>
+          <t>https://www.globenewswire.com/news-release/2024/03/06/2841834/0/en/Constellation-Software-Inc-Announces-Results-for-the-Fourth-Quarter-and-Year-Ended-December-31-2023-and-Declares-Quarterly-Dividend.html</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>acquisition_count</t>
+          <t>acquisitions_cash_spent</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>FY2008</t>
+          <t>FY2024</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>17</v>
+        <v>1792</v>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>count approximate</t>
+          <t>USD millions</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
@@ -6242,47 +6342,43 @@
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>https://www.mbi-deepdives.com/content/files/2022/07/Constellation-Software-SH-Letters-Merged.pdf</t>
-        </is>
-      </c>
-      <c r="G136" t="inlineStr">
-        <is>
-          <t>2008 letter: 'bought the Maximus assets and 16 other businesses' -&gt; 1 + 16 = 17.</t>
-        </is>
-      </c>
+          <t>https://www.globenewswire.com/news-release/2025/03/07/3039269/0/en/Constellation-Software-Inc-Announces-Results-for-the-Fourth-Quarter-and-Year-Ended-December-31-2024-and-Declares-Quarterly-Dividend.html</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>acquisition_count</t>
+          <t>acquisitions_cash_spent</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>FY2012</t>
+          <t>FY2025</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>35</v>
+        <v>1579</v>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>USD millions</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>derived</t>
+          <t>company</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1113678/000119312515138334/d906182dex26.htm</t>
+          <t>https://www.globenewswire.com/news-release/2026/03/09/3251696/0/en/constellation-software-inc-announces-results-for-the-fourth-quarter-and-year-ended-december-31-2025-and-declares-quarterly-dividend.html</t>
         </is>
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>Derived from a comparative sentence in the FY2013 disclosure ('thirty acquisitions... compared to thirty-five in 2012'); no primary FY2012 release figure found.</t>
+          <t>Total acquisition consideration of $1,579M including holdbacks and contingent consideration.</t>
         </is>
       </c>
     </row>
@@ -6294,15 +6390,15 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>FY2013</t>
+          <t>FY2008</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>count approximate</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
@@ -6312,10 +6408,14 @@
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1113678/000119312514275886/d757774dex21.htm</t>
-        </is>
-      </c>
-      <c r="G138" t="inlineStr"/>
+          <t>https://www.mbi-deepdives.com/content/files/2022/07/Constellation-Software-SH-Letters-Merged.pdf</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>2008 letter: 'bought the Maximus assets and 16 other businesses' -&gt; 1 + 16 = 17.</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -6325,11 +6425,11 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>FY2014</t>
+          <t>FY2012</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="D139" t="inlineStr">
         <is>
@@ -6338,7 +6438,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>company</t>
+          <t>derived</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
@@ -6348,7 +6448,7 @@
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>Lower than FY2013's 30; the intake's 'record year' framing for FY2014 acquisitions was not corroborated on a count or cash-consideration basis.</t>
+          <t>Derived from a comparative sentence in the FY2013 disclosure ('thirty acquisitions... compared to thirty-five in 2012'); no primary FY2012 release figure found.</t>
         </is>
       </c>
     </row>
@@ -6360,11 +6460,11 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>FY2015</t>
+          <t>FY2013</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="D140" t="inlineStr">
         <is>
@@ -6373,19 +6473,15 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>third_party</t>
+          <t>company</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>https://tracxn.com/d/acquisitions/acquisitions-by-constellation-software/__YaRluimuGqgVfqr0Xhgb2dPWiMKnmgzXPcPNPni5Ssg</t>
-        </is>
-      </c>
-      <c r="G140" t="inlineStr">
-        <is>
-          <t>Low-confidence third-party M&amp;A database count; implausibly low vs. the company's typical pace elsewhere in this window. Matches parent_long_run.</t>
-        </is>
-      </c>
+          <t>https://www.sec.gov/Archives/edgar/data/1113678/000119312514275886/d757774dex21.htm</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -6395,11 +6491,11 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>FY2019</t>
+          <t>FY2014</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>3</v>
+        <v>23</v>
       </c>
       <c r="D141" t="inlineStr">
         <is>
@@ -6408,17 +6504,17 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>third_party</t>
+          <t>company</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>https://nicoper.substack.com/p/4-constellation-acquisitions-2022</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1113678/000119312515138334/d906182dex26.htm</t>
         </is>
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>Third-party count; matches parent_long_run.</t>
+          <t>Lower than FY2013's 30; the intake's 'record year' framing for FY2014 acquisitions was not corroborated on a count or cash-consideration basis.</t>
         </is>
       </c>
     </row>
@@ -6430,85 +6526,79 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>FY2021</t>
-        </is>
-      </c>
-      <c r="C142" t="n">
-        <v>85</v>
+          <t>FY2015</t>
+        </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>count approximate, company-wide, stated as a minimum ('more than')</t>
+          <t>count</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>third_party</t>
+          <t>unreliable</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>https://explore.volarisgroup.com/volaris-group-blog/volaris-recognized-as-a-top-acquirer</t>
+          <t>https://tracxn.com/d/acquisitions/acquisitions-by-constellation-software/__YaRluimuGqgVfqr0Xhgb2dPWiMKnmgzXPcPNPni5Ssg</t>
         </is>
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>Third-party (Volaris/Corum Group) reporting; not a Constellation-disclosed figure.</t>
+          <t>Low-confidence third-party M&amp;A database count; implausibly low vs. the company's typical pace elsewhere in this window. Matches parent_long_run. Set to gap: counts disclosed major deals only, not the annual total.</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>shares_outstanding</t>
+          <t>acquisition_count</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>FY2023</t>
-        </is>
-      </c>
-      <c r="C143" t="n">
-        <v>21.19</v>
+          <t>FY2019</t>
+        </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>millions</t>
+          <t>count</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>third_party</t>
+          <t>unreliable</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>https://www.macrotrends.net/stocks/charts/CNSWF/constellation-software/shares-outstanding</t>
+          <t>https://nicoper.substack.com/p/4-constellation-acquisitions-2022</t>
         </is>
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>Matches ledger.json.</t>
+          <t>Third-party count; matches parent_long_run. Set to gap: counts disclosed major deals only, not the annual total.</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>shares_outstanding</t>
+          <t>acquisition_count</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>FY2024</t>
+          <t>FY2021</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>21.19</v>
+        <v>85</v>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>millions</t>
+          <t>count approximate, company-wide, stated as a minimum ('more than')</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
@@ -6518,12 +6608,12 @@
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>https://www.macrotrends.net/stocks/charts/CNSWF/constellation-software/shares-outstanding</t>
+          <t>https://explore.volarisgroup.com/volaris-group-blog/volaris-recognized-as-a-top-acquirer</t>
         </is>
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>Matches ledger.json.</t>
+          <t>Third-party (Volaris/Corum Group) reporting; not a Constellation-disclosed figure.</t>
         </is>
       </c>
     </row>
@@ -6535,7 +6625,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>FY2025</t>
+          <t>FY2023</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -6548,17 +6638,17 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>company</t>
+          <t>third_party</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2026/03/09/3251696/0/en/constellation-software-inc-announces-results-for-the-fourth-quarter-and-year-ended-december-31-2025-and-declares-quarterly-dividend.html</t>
+          <t>https://www.macrotrends.net/stocks/charts/CNSWF/constellation-software/shares-outstanding</t>
         </is>
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>21,191,530 shares per the company's FY2025 results release.</t>
+          <t>Matches ledger.json.</t>
         </is>
       </c>
     </row>
@@ -6570,7 +6660,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>FY2006</t>
+          <t>FY2024</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -6578,7 +6668,7 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>millions of shares, approximate, carried forward</t>
+          <t>millions</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
@@ -6588,12 +6678,12 @@
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>https://thequalityinvestor.substack.com/p/constellation-software-180x-in-less</t>
+          <t>https://www.macrotrends.net/stocks/charts/CNSWF/constellation-software/shares-outstanding</t>
         </is>
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>Assumption applied by Fable on 2026-09-14: the source states 21,191,530 shares outstanding, 'mostly unchanged since 2006' and 'has not grown since the IPO'; corroborated by https://www.marketscreener.com/quote/stock/CONSTELLATION-SOFTWARE-IN-1409607/news/Multibagger-Stories-Constellation-Software-44687508/. No company sourced year end count was found for FY2006. Per share figures for this year rest on this assumption and are labelled approximate.</t>
+          <t>Matches ledger.json.</t>
         </is>
       </c>
     </row>
@@ -6605,7 +6695,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>FY2007</t>
+          <t>FY2025</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -6613,22 +6703,22 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>millions of shares, approximate, carried forward</t>
+          <t>millions</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>third_party</t>
+          <t>company</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>https://thequalityinvestor.substack.com/p/constellation-software-180x-in-less</t>
+          <t>https://www.globenewswire.com/news-release/2026/03/09/3251696/0/en/constellation-software-inc-announces-results-for-the-fourth-quarter-and-year-ended-december-31-2025-and-declares-quarterly-dividend.html</t>
         </is>
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>Assumption applied by Fable on 2026-09-14: the source states 21,191,530 shares outstanding, 'mostly unchanged since 2006' and 'has not grown since the IPO'; corroborated by https://www.marketscreener.com/quote/stock/CONSTELLATION-SOFTWARE-IN-1409607/news/Multibagger-Stories-Constellation-Software-44687508/. No company sourced year end count was found for FY2007. Per share figures for this year rest on this assumption and are labelled approximate.</t>
+          <t>21,191,530 shares per the company's FY2025 results release.</t>
         </is>
       </c>
     </row>
@@ -6640,7 +6730,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>FY2008</t>
+          <t>FY2006</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -6663,7 +6753,7 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>Assumption applied by Fable on 2026-09-14: the source states 21,191,530 shares outstanding, 'mostly unchanged since 2006' and 'has not grown since the IPO'; corroborated by https://www.marketscreener.com/quote/stock/CONSTELLATION-SOFTWARE-IN-1409607/news/Multibagger-Stories-Constellation-Software-44687508/. No company sourced year end count was found for FY2008. Per share figures for this year rest on this assumption and are labelled approximate.</t>
+          <t>Assumption applied by Fable on 2026-09-14: the source states 21,191,530 shares outstanding, 'mostly unchanged since 2006' and 'has not grown since the IPO'; corroborated by https://www.marketscreener.com/quote/stock/CONSTELLATION-SOFTWARE-IN-1409607/news/Multibagger-Stories-Constellation-Software-44687508/. No company sourced year end count was found for FY2006. Per share figures for this year rest on this assumption and are labelled approximate.</t>
         </is>
       </c>
     </row>
@@ -6675,7 +6765,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>FY2009</t>
+          <t>FY2007</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -6698,7 +6788,7 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>Assumption applied by Fable on 2026-09-14: the source states 21,191,530 shares outstanding, 'mostly unchanged since 2006' and 'has not grown since the IPO'; corroborated by https://www.marketscreener.com/quote/stock/CONSTELLATION-SOFTWARE-IN-1409607/news/Multibagger-Stories-Constellation-Software-44687508/. No company sourced year end count was found for FY2009. Per share figures for this year rest on this assumption and are labelled approximate.</t>
+          <t>Assumption applied by Fable on 2026-09-14: the source states 21,191,530 shares outstanding, 'mostly unchanged since 2006' and 'has not grown since the IPO'; corroborated by https://www.marketscreener.com/quote/stock/CONSTELLATION-SOFTWARE-IN-1409607/news/Multibagger-Stories-Constellation-Software-44687508/. No company sourced year end count was found for FY2007. Per share figures for this year rest on this assumption and are labelled approximate.</t>
         </is>
       </c>
     </row>
@@ -6710,7 +6800,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>FY2010</t>
+          <t>FY2008</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -6733,7 +6823,7 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>Assumption applied by Fable on 2026-09-14: the source states 21,191,530 shares outstanding, 'mostly unchanged since 2006' and 'has not grown since the IPO'; corroborated by https://www.marketscreener.com/quote/stock/CONSTELLATION-SOFTWARE-IN-1409607/news/Multibagger-Stories-Constellation-Software-44687508/. No company sourced year end count was found for FY2010. Per share figures for this year rest on this assumption and are labelled approximate.</t>
+          <t>Assumption applied by Fable on 2026-09-14: the source states 21,191,530 shares outstanding, 'mostly unchanged since 2006' and 'has not grown since the IPO'; corroborated by https://www.marketscreener.com/quote/stock/CONSTELLATION-SOFTWARE-IN-1409607/news/Multibagger-Stories-Constellation-Software-44687508/. No company sourced year end count was found for FY2008. Per share figures for this year rest on this assumption and are labelled approximate.</t>
         </is>
       </c>
     </row>
@@ -6745,7 +6835,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>FY2011</t>
+          <t>FY2009</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -6768,7 +6858,7 @@
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>Assumption applied by Fable on 2026-09-14: the source states 21,191,530 shares outstanding, 'mostly unchanged since 2006' and 'has not grown since the IPO'; corroborated by https://www.marketscreener.com/quote/stock/CONSTELLATION-SOFTWARE-IN-1409607/news/Multibagger-Stories-Constellation-Software-44687508/. No company sourced year end count was found for FY2011. Per share figures for this year rest on this assumption and are labelled approximate.</t>
+          <t>Assumption applied by Fable on 2026-09-14: the source states 21,191,530 shares outstanding, 'mostly unchanged since 2006' and 'has not grown since the IPO'; corroborated by https://www.marketscreener.com/quote/stock/CONSTELLATION-SOFTWARE-IN-1409607/news/Multibagger-Stories-Constellation-Software-44687508/. No company sourced year end count was found for FY2009. Per share figures for this year rest on this assumption and are labelled approximate.</t>
         </is>
       </c>
     </row>
@@ -6780,7 +6870,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>FY2012</t>
+          <t>FY2010</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -6803,7 +6893,7 @@
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>Assumption applied by Fable on 2026-09-14: the source states 21,191,530 shares outstanding, 'mostly unchanged since 2006' and 'has not grown since the IPO'; corroborated by https://www.marketscreener.com/quote/stock/CONSTELLATION-SOFTWARE-IN-1409607/news/Multibagger-Stories-Constellation-Software-44687508/. No company sourced year end count was found for FY2012. Per share figures for this year rest on this assumption and are labelled approximate.</t>
+          <t>Assumption applied by Fable on 2026-09-14: the source states 21,191,530 shares outstanding, 'mostly unchanged since 2006' and 'has not grown since the IPO'; corroborated by https://www.marketscreener.com/quote/stock/CONSTELLATION-SOFTWARE-IN-1409607/news/Multibagger-Stories-Constellation-Software-44687508/. No company sourced year end count was found for FY2010. Per share figures for this year rest on this assumption and are labelled approximate.</t>
         </is>
       </c>
     </row>
@@ -6815,7 +6905,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>FY2013</t>
+          <t>FY2011</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -6838,7 +6928,7 @@
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>Assumption applied by Fable on 2026-09-14: the source states 21,191,530 shares outstanding, 'mostly unchanged since 2006' and 'has not grown since the IPO'; corroborated by https://www.marketscreener.com/quote/stock/CONSTELLATION-SOFTWARE-IN-1409607/news/Multibagger-Stories-Constellation-Software-44687508/. No company sourced year end count was found for FY2013. Per share figures for this year rest on this assumption and are labelled approximate.</t>
+          <t>Assumption applied by Fable on 2026-09-14: the source states 21,191,530 shares outstanding, 'mostly unchanged since 2006' and 'has not grown since the IPO'; corroborated by https://www.marketscreener.com/quote/stock/CONSTELLATION-SOFTWARE-IN-1409607/news/Multibagger-Stories-Constellation-Software-44687508/. No company sourced year end count was found for FY2011. Per share figures for this year rest on this assumption and are labelled approximate.</t>
         </is>
       </c>
     </row>
@@ -6850,7 +6940,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>FY2014</t>
+          <t>FY2012</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -6873,7 +6963,7 @@
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>Assumption applied by Fable on 2026-09-14: the source states 21,191,530 shares outstanding, 'mostly unchanged since 2006' and 'has not grown since the IPO'; corroborated by https://www.marketscreener.com/quote/stock/CONSTELLATION-SOFTWARE-IN-1409607/news/Multibagger-Stories-Constellation-Software-44687508/. No company sourced year end count was found for FY2014. Per share figures for this year rest on this assumption and are labelled approximate.</t>
+          <t>Assumption applied by Fable on 2026-09-14: the source states 21,191,530 shares outstanding, 'mostly unchanged since 2006' and 'has not grown since the IPO'; corroborated by https://www.marketscreener.com/quote/stock/CONSTELLATION-SOFTWARE-IN-1409607/news/Multibagger-Stories-Constellation-Software-44687508/. No company sourced year end count was found for FY2012. Per share figures for this year rest on this assumption and are labelled approximate.</t>
         </is>
       </c>
     </row>
@@ -6885,7 +6975,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>FY2015</t>
+          <t>FY2013</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -6908,7 +6998,7 @@
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>Assumption applied by Fable on 2026-09-14: the source states 21,191,530 shares outstanding, 'mostly unchanged since 2006' and 'has not grown since the IPO'; corroborated by https://www.marketscreener.com/quote/stock/CONSTELLATION-SOFTWARE-IN-1409607/news/Multibagger-Stories-Constellation-Software-44687508/. No company sourced year end count was found for FY2015. Per share figures for this year rest on this assumption and are labelled approximate.</t>
+          <t>Assumption applied by Fable on 2026-09-14: the source states 21,191,530 shares outstanding, 'mostly unchanged since 2006' and 'has not grown since the IPO'; corroborated by https://www.marketscreener.com/quote/stock/CONSTELLATION-SOFTWARE-IN-1409607/news/Multibagger-Stories-Constellation-Software-44687508/. No company sourced year end count was found for FY2013. Per share figures for this year rest on this assumption and are labelled approximate.</t>
         </is>
       </c>
     </row>
@@ -6920,7 +7010,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>FY2016</t>
+          <t>FY2014</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -6943,7 +7033,7 @@
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>Assumption applied by Fable on 2026-09-14: the source states 21,191,530 shares outstanding, 'mostly unchanged since 2006' and 'has not grown since the IPO'; corroborated by https://www.marketscreener.com/quote/stock/CONSTELLATION-SOFTWARE-IN-1409607/news/Multibagger-Stories-Constellation-Software-44687508/. No company sourced year end count was found for FY2016. Per share figures for this year rest on this assumption and are labelled approximate.</t>
+          <t>Assumption applied by Fable on 2026-09-14: the source states 21,191,530 shares outstanding, 'mostly unchanged since 2006' and 'has not grown since the IPO'; corroborated by https://www.marketscreener.com/quote/stock/CONSTELLATION-SOFTWARE-IN-1409607/news/Multibagger-Stories-Constellation-Software-44687508/. No company sourced year end count was found for FY2014. Per share figures for this year rest on this assumption and are labelled approximate.</t>
         </is>
       </c>
     </row>
@@ -6955,7 +7045,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>FY2017</t>
+          <t>FY2015</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -6978,7 +7068,7 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>Assumption applied by Fable on 2026-09-14: the source states 21,191,530 shares outstanding, 'mostly unchanged since 2006' and 'has not grown since the IPO'; corroborated by https://www.marketscreener.com/quote/stock/CONSTELLATION-SOFTWARE-IN-1409607/news/Multibagger-Stories-Constellation-Software-44687508/. No company sourced year end count was found for FY2017. Per share figures for this year rest on this assumption and are labelled approximate.</t>
+          <t>Assumption applied by Fable on 2026-09-14: the source states 21,191,530 shares outstanding, 'mostly unchanged since 2006' and 'has not grown since the IPO'; corroborated by https://www.marketscreener.com/quote/stock/CONSTELLATION-SOFTWARE-IN-1409607/news/Multibagger-Stories-Constellation-Software-44687508/. No company sourced year end count was found for FY2015. Per share figures for this year rest on this assumption and are labelled approximate.</t>
         </is>
       </c>
     </row>
@@ -6990,7 +7080,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>FY2018</t>
+          <t>FY2016</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -7013,7 +7103,7 @@
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>Assumption applied by Fable on 2026-09-14: the source states 21,191,530 shares outstanding, 'mostly unchanged since 2006' and 'has not grown since the IPO'; corroborated by https://www.marketscreener.com/quote/stock/CONSTELLATION-SOFTWARE-IN-1409607/news/Multibagger-Stories-Constellation-Software-44687508/. No company sourced year end count was found for FY2018. Per share figures for this year rest on this assumption and are labelled approximate.</t>
+          <t>Assumption applied by Fable on 2026-09-14: the source states 21,191,530 shares outstanding, 'mostly unchanged since 2006' and 'has not grown since the IPO'; corroborated by https://www.marketscreener.com/quote/stock/CONSTELLATION-SOFTWARE-IN-1409607/news/Multibagger-Stories-Constellation-Software-44687508/. No company sourced year end count was found for FY2016. Per share figures for this year rest on this assumption and are labelled approximate.</t>
         </is>
       </c>
     </row>
@@ -7025,7 +7115,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>FY2019</t>
+          <t>FY2017</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -7048,7 +7138,7 @@
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>Assumption applied by Fable on 2026-09-14: the source states 21,191,530 shares outstanding, 'mostly unchanged since 2006' and 'has not grown since the IPO'; corroborated by https://www.marketscreener.com/quote/stock/CONSTELLATION-SOFTWARE-IN-1409607/news/Multibagger-Stories-Constellation-Software-44687508/. No company sourced year end count was found for FY2019. Per share figures for this year rest on this assumption and are labelled approximate.</t>
+          <t>Assumption applied by Fable on 2026-09-14: the source states 21,191,530 shares outstanding, 'mostly unchanged since 2006' and 'has not grown since the IPO'; corroborated by https://www.marketscreener.com/quote/stock/CONSTELLATION-SOFTWARE-IN-1409607/news/Multibagger-Stories-Constellation-Software-44687508/. No company sourced year end count was found for FY2017. Per share figures for this year rest on this assumption and are labelled approximate.</t>
         </is>
       </c>
     </row>
@@ -7060,7 +7150,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>FY2020</t>
+          <t>FY2018</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -7083,7 +7173,7 @@
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>Assumption applied by Fable on 2026-09-14: the source states 21,191,530 shares outstanding, 'mostly unchanged since 2006' and 'has not grown since the IPO'; corroborated by https://www.marketscreener.com/quote/stock/CONSTELLATION-SOFTWARE-IN-1409607/news/Multibagger-Stories-Constellation-Software-44687508/. No company sourced year end count was found for FY2020. Per share figures for this year rest on this assumption and are labelled approximate.</t>
+          <t>Assumption applied by Fable on 2026-09-14: the source states 21,191,530 shares outstanding, 'mostly unchanged since 2006' and 'has not grown since the IPO'; corroborated by https://www.marketscreener.com/quote/stock/CONSTELLATION-SOFTWARE-IN-1409607/news/Multibagger-Stories-Constellation-Software-44687508/. No company sourced year end count was found for FY2018. Per share figures for this year rest on this assumption and are labelled approximate.</t>
         </is>
       </c>
     </row>
@@ -7095,7 +7185,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>FY2021</t>
+          <t>FY2019</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -7118,7 +7208,7 @@
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>Assumption applied by Fable on 2026-09-14: the source states 21,191,530 shares outstanding, 'mostly unchanged since 2006' and 'has not grown since the IPO'; corroborated by https://www.marketscreener.com/quote/stock/CONSTELLATION-SOFTWARE-IN-1409607/news/Multibagger-Stories-Constellation-Software-44687508/. No company sourced year end count was found for FY2021. Per share figures for this year rest on this assumption and are labelled approximate.</t>
+          <t>Assumption applied by Fable on 2026-09-14: the source states 21,191,530 shares outstanding, 'mostly unchanged since 2006' and 'has not grown since the IPO'; corroborated by https://www.marketscreener.com/quote/stock/CONSTELLATION-SOFTWARE-IN-1409607/news/Multibagger-Stories-Constellation-Software-44687508/. No company sourced year end count was found for FY2019. Per share figures for this year rest on this assumption and are labelled approximate.</t>
         </is>
       </c>
     </row>
@@ -7130,7 +7220,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>FY2022</t>
+          <t>FY2020</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -7153,62 +7243,62 @@
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>Assumption applied by Fable on 2026-09-14: the source states 21,191,530 shares outstanding, 'mostly unchanged since 2006' and 'has not grown since the IPO'; corroborated by https://www.marketscreener.com/quote/stock/CONSTELLATION-SOFTWARE-IN-1409607/news/Multibagger-Stories-Constellation-Software-44687508/. No company sourced year end count was found for FY2022. Per share figures for this year rest on this assumption and are labelled approximate.</t>
+          <t>Assumption applied by Fable on 2026-09-14: the source states 21,191,530 shares outstanding, 'mostly unchanged since 2006' and 'has not grown since the IPO'; corroborated by https://www.marketscreener.com/quote/stock/CONSTELLATION-SOFTWARE-IN-1409607/news/Multibagger-Stories-Constellation-Software-44687508/. No company sourced year end count was found for FY2020. Per share figures for this year rest on this assumption and are labelled approximate.</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>dividends_per_share_regular</t>
+          <t>shares_outstanding</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>FY2010</t>
+          <t>FY2021</t>
         </is>
       </c>
       <c r="C163" t="n">
-        <v>2</v>
+        <v>21.19</v>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>CAD per share approximate</t>
+          <t>millions of shares, approximate, carried forward</t>
         </is>
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>company</t>
+          <t>third_party</t>
         </is>
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>https://www.csisoftware.com/docs/default-source/press-releases/q4_2010_press_release.pdf</t>
+          <t>https://thequalityinvestor.substack.com/p/constellation-software-180x-in-less</t>
         </is>
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>Dividend declared March 2, 2011 for FY2010; currency assumed CAD (TSX-listed shares), not directly confirmed from the release text. Whether styled 'annual' or an aggregate of quarterly payments was not confirmed.</t>
+          <t>Assumption applied by Fable on 2026-09-14: the source states 21,191,530 shares outstanding, 'mostly unchanged since 2006' and 'has not grown since the IPO'; corroborated by https://www.marketscreener.com/quote/stock/CONSTELLATION-SOFTWARE-IN-1409607/news/Multibagger-Stories-Constellation-Software-44687508/. No company sourced year end count was found for FY2021. Per share figures for this year rest on this assumption and are labelled approximate.</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>dividends_per_share_regular</t>
+          <t>shares_outstanding</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>FY2011</t>
+          <t>FY2022</t>
         </is>
       </c>
       <c r="C164" t="n">
-        <v>2</v>
+        <v>21.19</v>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>CAD per share approximate</t>
+          <t>millions of shares, approximate, carried forward</t>
         </is>
       </c>
       <c r="E164" t="inlineStr">
@@ -7218,12 +7308,12 @@
       </c>
       <c r="F164" t="inlineStr">
         <is>
-          <t>https://businesscaseweekly.substack.com/p/bcw-49-constellation-software</t>
+          <t>https://thequalityinvestor.substack.com/p/constellation-software-180x-in-less</t>
         </is>
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>'$2 a share for 2011 in total', before the board adopted a true $1/share quarterly dividend starting Q1 2012.</t>
+          <t>Assumption applied by Fable on 2026-09-14: the source states 21,191,530 shares outstanding, 'mostly unchanged since 2006' and 'has not grown since the IPO'; corroborated by https://www.marketscreener.com/quote/stock/CONSTELLATION-SOFTWARE-IN-1409607/news/Multibagger-Stories-Constellation-Software-44687508/. No company sourced year end count was found for FY2022. Per share figures for this year rest on this assumption and are labelled approximate.</t>
         </is>
       </c>
     </row>
@@ -7235,15 +7325,15 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>FY2013</t>
+          <t>FY2010</t>
         </is>
       </c>
       <c r="C165" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>USD (4 x USD 1.00 quarterly)</t>
+          <t>CAD per share approximate</t>
         </is>
       </c>
       <c r="E165" t="inlineStr">
@@ -7253,12 +7343,12 @@
       </c>
       <c r="F165" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2013/10/30/1474983/0/en/Constellation-Software-Inc-Announces-Results-for-the-Third-Quarter-Ended-September-30-2013-and-Declares-Quarterly-Dividend.html</t>
+          <t>https://www.csisoftware.com/docs/default-source/press-releases/q4_2010_press_release.pdf</t>
         </is>
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>Quarterly rate of USD 1.00 confirmed; annual total assumes the same rate held for all four quarters of FY2013 (unchanged since 2012 per company disclosure pattern).</t>
+          <t>Dividend declared March 2, 2011 for FY2010; currency assumed CAD (TSX-listed shares), not directly confirmed from the release text. Whether styled 'annual' or an aggregate of quarterly payments was not confirmed.</t>
         </is>
       </c>
     </row>
@@ -7270,28 +7360,32 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>FY2014</t>
+          <t>FY2011</t>
         </is>
       </c>
       <c r="C166" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>USD (4 x USD 1.00 quarterly)</t>
+          <t>CAD per share approximate</t>
         </is>
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>company</t>
+          <t>third_party</t>
         </is>
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2014/03/06/1475011/0/en/Constellation-Software-Inc-Declares-Quarterly-Dividend.html</t>
-        </is>
-      </c>
-      <c r="G166" t="inlineStr"/>
+          <t>https://businesscaseweekly.substack.com/p/bcw-49-constellation-software</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>'$2 a share for 2011 in total', before the board adopted a true $1/share quarterly dividend starting Q1 2012.</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -7301,7 +7395,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>FY2015</t>
+          <t>FY2013</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -7319,12 +7413,12 @@
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2016/02/17/1061530/0/en/Constellation-Software-Inc-Announces-Results-for-the-Fourth-Quarter-and-Year-Ended-December-31-2015-and-Declares-Quarterly-Dividend.html</t>
+          <t>https://www.globenewswire.com/news-release/2013/10/30/1474983/0/en/Constellation-Software-Inc-Announces-Results-for-the-Third-Quarter-Ended-September-30-2013-and-Declares-Quarterly-Dividend.html</t>
         </is>
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>No special dividend named in this release for FY2015.</t>
+          <t>Quarterly rate of USD 1.00 confirmed; annual total assumes the same rate held for all four quarters of FY2013 (unchanged since 2012 per company disclosure pattern).</t>
         </is>
       </c>
     </row>
@@ -7336,7 +7430,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>FY2018</t>
+          <t>FY2014</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -7354,14 +7448,10 @@
       </c>
       <c r="F168" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2019/02/14/1725078/0/en/Constellation-Software-Inc-Announces-Results-for-the-Fourth-Quarter-and-Year-Ended-December-31-2018-and-Declares-Quarterly-and-Special-Dividends.html</t>
-        </is>
-      </c>
-      <c r="G168" t="inlineStr">
-        <is>
-          <t>Declared alongside the USD 20.00 special dividend.</t>
-        </is>
-      </c>
+          <t>https://www.globenewswire.com/news-release/2014/03/06/1475011/0/en/Constellation-Software-Inc-Declares-Quarterly-Dividend.html</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -7371,7 +7461,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>FY2019</t>
+          <t>FY2015</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -7389,10 +7479,14 @@
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2020/02/13/1984977/0/en/Constellation-Software-Inc-Announces-Results-for-the-Fourth-Quarter-and-Year-Ended-December-31-2019-and-Declares-Quarterly-Dividend.html</t>
-        </is>
-      </c>
-      <c r="G169" t="inlineStr"/>
+          <t>https://www.globenewswire.com/news-release/2016/02/17/1061530/0/en/Constellation-Software-Inc-Announces-Results-for-the-Fourth-Quarter-and-Year-Ended-December-31-2015-and-Declares-Quarterly-Dividend.html</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>No special dividend named in this release for FY2015.</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -7402,7 +7496,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>FY2020</t>
+          <t>FY2018</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -7420,10 +7514,14 @@
       </c>
       <c r="F170" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2020/11/02/2118890/0/en/Constellation-Software-Inc-Announces-Results-for-the-Third-Quarter-Ended-September-30-2020-and-Declares-Quarterly-Dividend.html</t>
-        </is>
-      </c>
-      <c r="G170" t="inlineStr"/>
+          <t>https://www.globenewswire.com/news-release/2019/02/14/1725078/0/en/Constellation-Software-Inc-Announces-Results-for-the-Fourth-Quarter-and-Year-Ended-December-31-2018-and-Declares-Quarterly-and-Special-Dividends.html</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>Declared alongside the USD 20.00 special dividend.</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -7433,7 +7531,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>FY2022</t>
+          <t>FY2019</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -7451,14 +7549,10 @@
       </c>
       <c r="F171" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2023/03/29/2637195/0/en/Constellation-Software-Inc-Announces-Results-for-the-Fourth-Quarter-and-Year-Ended-December-31-2022-and-Declares-Quarterly-Dividend.html</t>
-        </is>
-      </c>
-      <c r="G171" t="inlineStr">
-        <is>
-          <t>No special dividend named in this release.</t>
-        </is>
-      </c>
+          <t>https://www.globenewswire.com/news-release/2020/02/13/1984977/0/en/Constellation-Software-Inc-Announces-Results-for-the-Fourth-Quarter-and-Year-Ended-December-31-2019-and-Declares-Quarterly-Dividend.html</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -7468,7 +7562,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>FY2023</t>
+          <t>FY2020</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -7486,7 +7580,7 @@
       </c>
       <c r="F172" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2024/3/6/2841834/0/en/Constellation-Software-Inc-Announces-Results-for-the-Fourth-Quarter-and-Year-Ended-December-31-2023-and-Declares-Quarterly-Dividend.html</t>
+          <t>https://www.globenewswire.com/news-release/2020/11/02/2118890/0/en/Constellation-Software-Inc-Announces-Results-for-the-Third-Quarter-Ended-September-30-2020-and-Declares-Quarterly-Dividend.html</t>
         </is>
       </c>
       <c r="G172" t="inlineStr"/>
@@ -7499,7 +7593,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>FY2024</t>
+          <t>FY2022</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -7517,10 +7611,14 @@
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2025/03/07/3039269/0/en/Constellation-Software-Inc-Announces-Results-for-the-Fourth-Quarter-and-Year-Ended-December-31-2024-and-Declares-Quarterly-Dividend.html</t>
-        </is>
-      </c>
-      <c r="G173" t="inlineStr"/>
+          <t>https://www.globenewswire.com/news-release/2023/03/29/2637195/0/en/Constellation-Software-Inc-Announces-Results-for-the-Fourth-Quarter-and-Year-Ended-December-31-2022-and-Declares-Quarterly-Dividend.html</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>No special dividend named in this release.</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -7530,7 +7628,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>FY2025</t>
+          <t>FY2023</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -7548,32 +7646,28 @@
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2026/03/09/3251696/0/en/constellation-software-inc-announces-results-for-the-fourth-quarter-and-year-ended-december-31-2025-and-declares-quarterly-dividend.html</t>
-        </is>
-      </c>
-      <c r="G174" t="inlineStr">
-        <is>
-          <t>Regular rate still USD 1.00 quarterly; no special dividend named.</t>
-        </is>
-      </c>
+          <t>https://www.globenewswire.com/news-release/2024/3/6/2841834/0/en/Constellation-Software-Inc-Announces-Results-for-the-Fourth-Quarter-and-Year-Ended-December-31-2023-and-Declares-Quarterly-Dividend.html</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>dividends_per_share_special</t>
+          <t>dividends_per_share_regular</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>FY2018</t>
+          <t>FY2024</t>
         </is>
       </c>
       <c r="C175" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>USD per share, one-time special dividend</t>
+          <t>USD (4 x USD 1.00 quarterly)</t>
         </is>
       </c>
       <c r="E175" t="inlineStr">
@@ -7583,32 +7677,28 @@
       </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2019/02/14/1725078/0/en/Constellation-Software-Inc-Announces-Results-for-the-Fourth-Quarter-and-Year-Ended-December-31-2018-and-Declares-Quarterly-and-Special-Dividends.html</t>
-        </is>
-      </c>
-      <c r="G175" t="inlineStr">
-        <is>
-          <t>Declared February 14, 2019 alongside FY2018 results and the regular USD 1.00 quarterly dividend, both paid April 5, 2019 to holders of record March 16, 2019. Company: 'we have capital in excess of our needs and should return the excess to shareholders.' Known issue 8: this is the only special dividend found anywhere across all five stage1 sweeps; earlier years were specifically searched and none were found -- see coverage note.</t>
-        </is>
-      </c>
+          <t>https://www.globenewswire.com/news-release/2025/03/07/3039269/0/en/Constellation-Software-Inc-Announces-Results-for-the-Fourth-Quarter-and-Year-Ended-December-31-2024-and-Declares-Quarterly-Dividend.html</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>employees</t>
+          <t>dividends_per_share_regular</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>FY2011</t>
+          <t>FY2025</t>
         </is>
       </c>
       <c r="C176" t="n">
-        <v>1022</v>
+        <v>4</v>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>count (R&amp;D employees only, NOT total company headcount)</t>
+          <t>USD (4 x USD 1.00 quarterly)</t>
         </is>
       </c>
       <c r="E176" t="inlineStr">
@@ -7618,177 +7708,189 @@
       </c>
       <c r="F176" t="inlineStr">
         <is>
-          <t>https://www.csisoftware.com/docs/default-source/investor-relations/statutory-filings/csu-2011-aif.pdf</t>
+          <t>https://www.globenewswire.com/news-release/2026/03/09/3251696/0/en/constellation-software-inc-announces-results-for-the-fourth-quarter-and-year-ended-december-31-2025-and-declares-quarterly-dividend.html</t>
         </is>
       </c>
       <c r="G176" t="inlineStr">
         <is>
-          <t>2011 AIF: ~1,022 employees involved in R&amp;D for fiscal 2011. This is an R&amp;D headcount subset; no total company-wide employee figure was found for FY2011.</t>
+          <t>Regular rate still USD 1.00 quarterly; no special dividend named.</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>employees</t>
+          <t>dividends_per_share_regular</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>FY2015</t>
+          <t>FY2012</t>
         </is>
       </c>
       <c r="C177" t="n">
-        <v>9924</v>
+        <v>4</v>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>average full-time employees (annual average)</t>
+          <t>USD (4 x USD 1.00 quarterly), derived</t>
         </is>
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>company</t>
+          <t>derived</t>
         </is>
       </c>
       <c r="F177" t="inlineStr">
         <is>
-          <t>https://www.csisoftware.com/wp-content/uploads/2026/04/2015-annual-information-form-final.pdf</t>
+          <t>https://www.globenewswire.com/news-release/2019/02/14/1725078/0/en/Constellation-Software-Inc-Announces-Results-for-the-Fourth-Quarter-and-Year-Ended-December-31-2018-and-Declares-Quarterly-and-Special-Dividends.html</t>
         </is>
       </c>
       <c r="G177" t="inlineStr">
         <is>
-          <t>2015 AIF: ~9,924 FTE average for fiscal 2015. A point-in-time figure of ~10,478 as at Dec 31, 2015 is also in the same source (different measurement basis, not a conflict).</t>
+          <t>Not individually sourced for FY2012. The quarterly rate of USD 1.00 is company sourced for FY2013 to FY2015 and FY2018 to FY2020 and FY2022 to FY2025 with no change announced; carried as 4.00 for FY2012 by Fable review 2026-09-14 and labelled derived.</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>employees</t>
+          <t>dividends_per_share_regular</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>FY2019</t>
+          <t>FY2016</t>
         </is>
       </c>
       <c r="C178" t="n">
-        <v>23000</v>
+        <v>4</v>
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>approximate full-time employees, as at Dec 31 2019</t>
+          <t>USD (4 x USD 1.00 quarterly), derived</t>
         </is>
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>company</t>
+          <t>derived</t>
         </is>
       </c>
       <c r="F178" t="inlineStr">
         <is>
-          <t>https://www.csisoftware.com/docs/default-source/investor-relations/statutory-filings/2019-annual-information-form---final.pdf</t>
-        </is>
-      </c>
-      <c r="G178" t="inlineStr"/>
+          <t>https://www.globenewswire.com/news-release/2019/02/14/1725078/0/en/Constellation-Software-Inc-Announces-Results-for-the-Fourth-Quarter-and-Year-Ended-December-31-2018-and-Declares-Quarterly-and-Special-Dividends.html</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>Not individually sourced for FY2016. The quarterly rate of USD 1.00 is company sourced for FY2013 to FY2015 and FY2018 to FY2020 and FY2022 to FY2025 with no change announced; carried as 4.00 for FY2016 by Fable review 2026-09-14 and labelled derived.</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>employees</t>
+          <t>dividends_per_share_regular</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>FY2022</t>
+          <t>FY2017</t>
         </is>
       </c>
       <c r="C179" t="n">
-        <v>41000</v>
+        <v>4</v>
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>approximate full-time employees, globally</t>
+          <t>USD (4 x USD 1.00 quarterly), derived</t>
         </is>
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>company</t>
+          <t>derived</t>
         </is>
       </c>
       <c r="F179" t="inlineStr">
         <is>
-          <t>https://www.csisoftware.com/docs/default-source/investor-relations/2022-agm/csi-2021-mic-en.pdf</t>
+          <t>https://www.globenewswire.com/news-release/2019/02/14/1725078/0/en/Constellation-Software-Inc-Announces-Results-for-the-Fourth-Quarter-and-Year-Ended-December-31-2018-and-Declares-Quarterly-and-Special-Dividends.html</t>
         </is>
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>Known issue 7: company AIF-sourced figure of ~41,000 preferred over a third-party (macrotrends) figure of 45,000 as at Dec 31, 2022, which is recorded as a conflict.</t>
+          <t>Not individually sourced for FY2017. The quarterly rate of USD 1.00 is company sourced for FY2013 to FY2015 and FY2018 to FY2020 and FY2022 to FY2025 with no change announced; carried as 4.00 for FY2017 by Fable review 2026-09-14 and labelled derived.</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>employees</t>
+          <t>dividends_per_share_regular</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>FY2023</t>
+          <t>FY2021</t>
         </is>
       </c>
       <c r="C180" t="n">
-        <v>57637</v>
+        <v>4</v>
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>count, approximate (workforce-analytics estimate, not company-disclosed)</t>
+          <t>USD (4 x USD 1.00 quarterly), derived</t>
         </is>
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>third_party</t>
+          <t>derived</t>
         </is>
       </c>
       <c r="F180" t="inlineStr">
         <is>
-          <t>https://www.reveliolabs.com/companies/constellation-software/employees/</t>
-        </is>
-      </c>
-      <c r="G180" t="inlineStr"/>
+          <t>https://www.globenewswire.com/news-release/2019/02/14/1725078/0/en/Constellation-Software-Inc-Announces-Results-for-the-Fourth-Quarter-and-Year-Ended-December-31-2018-and-Declares-Quarterly-and-Special-Dividends.html</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>Not individually sourced for FY2021. The quarterly rate of USD 1.00 is company sourced for FY2013 to FY2015 and FY2018 to FY2020 and FY2022 to FY2025 with no change announced; carried as 4.00 for FY2021 by Fable review 2026-09-14 and labelled derived.</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>employees</t>
+          <t>dividends_per_share_special</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>FY2024</t>
+          <t>FY2018</t>
         </is>
       </c>
       <c r="C181" t="n">
-        <v>57217</v>
+        <v>20</v>
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>count, approximate (workforce-analytics estimate, not company-disclosed)</t>
+          <t>USD per share, one-time special dividend</t>
         </is>
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>third_party</t>
+          <t>company</t>
         </is>
       </c>
       <c r="F181" t="inlineStr">
         <is>
-          <t>https://www.reveliolabs.com/companies/constellation-software/employees/</t>
-        </is>
-      </c>
-      <c r="G181" t="inlineStr"/>
+          <t>https://www.globenewswire.com/news-release/2019/02/14/1725078/0/en/Constellation-Software-Inc-Announces-Results-for-the-Fourth-Quarter-and-Year-Ended-December-31-2018-and-Declares-Quarterly-and-Special-Dividends.html</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>Declared February 14, 2019 alongside FY2018 results and the regular USD 1.00 quarterly dividend, both paid April 5, 2019 to holders of record March 16, 2019. Company: 'we have capital in excess of our needs and should return the excess to shareholders.' Known issue 8: this is the only special dividend found anywhere across all five stage1 sweeps; earlier years were specifically searched and none were found -- see coverage note.</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -7798,50 +7900,50 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>FY2025</t>
+          <t>FY2011</t>
         </is>
       </c>
       <c r="C182" t="n">
-        <v>55775</v>
+        <v>1022</v>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>count, approximate (workforce-analytics estimate, not company-disclosed)</t>
+          <t>count (R&amp;D employees only, NOT total company headcount)</t>
         </is>
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>third_party</t>
+          <t>company</t>
         </is>
       </c>
       <c r="F182" t="inlineStr">
         <is>
-          <t>https://www.reveliolabs.com/companies/constellation-software/employees/</t>
+          <t>https://www.csisoftware.com/docs/default-source/investor-relations/statutory-filings/csu-2011-aif.pdf</t>
         </is>
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>Down 2.6%/-1,442 from FY2024 per the same aggregator.</t>
+          <t>2011 AIF: ~1,022 employees involved in R&amp;D for fiscal 2011. This is an R&amp;D headcount subset; no total company-wide employee figure was found for FY2011.</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>roic_pct</t>
+          <t>employees</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>FY2009</t>
+          <t>FY2015</t>
         </is>
       </c>
       <c r="C183" t="n">
-        <v>24</v>
+        <v>9924</v>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>percent</t>
+          <t>average full-time employees (annual average)</t>
         </is>
       </c>
       <c r="E183" t="inlineStr">
@@ -7851,32 +7953,32 @@
       </c>
       <c r="F183" t="inlineStr">
         <is>
-          <t>https://www.csisoftware.com/docs/default-source/investor-relations/presidents-letter/shareholder-letter---2009.pdf</t>
+          <t>https://www.csisoftware.com/wp-content/uploads/2026/04/2015-annual-information-form-final.pdf</t>
         </is>
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t>2009 President's letter reported 24% ROIC for 2009.</t>
+          <t>2015 AIF: ~9,924 FTE average for fiscal 2015. A point-in-time figure of ~10,478 as at Dec 31, 2015 is also in the same source (different measurement basis, not a conflict).</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>roic_pct</t>
+          <t>employees</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>FY2010</t>
+          <t>FY2019</t>
         </is>
       </c>
       <c r="C184" t="n">
-        <v>25</v>
+        <v>23000</v>
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>percent</t>
+          <t>approximate full-time employees, as at Dec 31 2019</t>
         </is>
       </c>
       <c r="E184" t="inlineStr">
@@ -7886,54 +7988,50 @@
       </c>
       <c r="F184" t="inlineStr">
         <is>
-          <t>https://www.csisoftware.com/docs/default-source/investor-relations/presidents-letter/shareholder-letter---2010.pdf</t>
-        </is>
-      </c>
-      <c r="G184" t="inlineStr">
-        <is>
-          <t>Reused from long-term-hold/holdings.json parent_long_run.</t>
-        </is>
-      </c>
+          <t>https://www.csisoftware.com/docs/default-source/investor-relations/statutory-filings/2019-annual-information-form---final.pdf</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>roic_plus_organic_pct</t>
+          <t>employees</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>FY2017</t>
+          <t>FY2022</t>
         </is>
       </c>
       <c r="C185" t="n">
-        <v>33</v>
+        <v>41000</v>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>percent, approximate</t>
+          <t>approximate full-time employees, globally</t>
         </is>
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>third_party</t>
+          <t>company</t>
         </is>
       </c>
       <c r="F185" t="inlineStr">
         <is>
-          <t>https://uploads-ssl.webflow.com/60e3655ca778911eb64b2a00/60f0777ead89beba9c51c0b3_Constellation-Software-Inc.-Shareholder-Letters.pdf</t>
+          <t>https://www.csisoftware.com/docs/default-source/investor-relations/2022-agm/csi-2021-mic-en.pdf</t>
         </is>
       </c>
       <c r="G185" t="inlineStr">
         <is>
-          <t>ROIC+OGr 'remained relatively flat at 33%' in 2017 with shareholders' Average Invested Capital growing 29%. Corroborated by a second third-party source (bizalmanac.substack.com) citing the same 33% figure and 29% ROIC alone for FY2017.</t>
+          <t>Known issue 7: company AIF-sourced figure of ~41,000 preferred over a third-party (macrotrends) figure of 45,000 as at Dec 31, 2022, which is recorded as a conflict.</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>capex</t>
+          <t>employees</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -7942,11 +8040,11 @@
         </is>
       </c>
       <c r="C186" t="n">
-        <v>68</v>
+        <v>57637</v>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>USD millions, approximate</t>
+          <t>count, approximate (workforce-analytics estimate, not company-disclosed)</t>
         </is>
       </c>
       <c r="E186" t="inlineStr">
@@ -7956,19 +8054,15 @@
       </c>
       <c r="F186" t="inlineStr">
         <is>
-          <t>https://www.stockopedia.com/share-prices/constellation-software-TSE:CSU/cashflow/</t>
-        </is>
-      </c>
-      <c r="G186" t="inlineStr">
-        <is>
-          <t>Aggregator-derived cash-flow-statement figure; not located in a company press release.</t>
-        </is>
-      </c>
+          <t>https://www.reveliolabs.com/companies/constellation-software/employees/</t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>capex</t>
+          <t>employees</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -7977,11 +8071,11 @@
         </is>
       </c>
       <c r="C187" t="n">
-        <v>72</v>
+        <v>57217</v>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>USD millions, approximate</t>
+          <t>count, approximate (workforce-analytics estimate, not company-disclosed)</t>
         </is>
       </c>
       <c r="E187" t="inlineStr">
@@ -7991,32 +8085,28 @@
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>https://www.stockopedia.com/share-prices/constellation-software-TSE:CSU/cashflow/</t>
-        </is>
-      </c>
-      <c r="G187" t="inlineStr">
-        <is>
-          <t>Aggregator-derived cash-flow-statement figure; not located in a company press release.</t>
-        </is>
-      </c>
+          <t>https://www.reveliolabs.com/companies/constellation-software/employees/</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>share_price_cad_year_end</t>
+          <t>employees</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>IPO 2006-05-17</t>
+          <t>FY2025</t>
         </is>
       </c>
       <c r="C188" t="n">
-        <v>17</v>
+        <v>55775</v>
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>CAD, IPO offering price (not a fiscal year-end close)</t>
+          <t>count, approximate (workforce-analytics estimate, not company-disclosed)</t>
         </is>
       </c>
       <c r="E188" t="inlineStr">
@@ -8026,94 +8116,102 @@
       </c>
       <c r="F188" t="inlineStr">
         <is>
-          <t>https://www.cantechletter.com/2025/05/constellation-software-has-delivered-a-36000-return-since-its-ipo-is-it-still-a-buy/</t>
+          <t>https://www.reveliolabs.com/companies/constellation-software/employees/</t>
         </is>
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>Constellation listed on the TSX May 17, 2006 at an IPO price of C$17.00/share (first-day close C$18.30). Not independently confirmed from Constellation's own short-form prospectus (WebFetch unavailable); treated as third_party. No FY2006-FY2025 fiscal year-end closing price could be sourced via WebSearch in any of the five intake sweeps -- year end prices are gap for every one of the 19 fiscal years, per known issue 9.</t>
+          <t>Down 2.6%/-1,442 from FY2024 per the same aggregator.</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>aggregate_returns</t>
+          <t>roic_pct</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>total_return_10yr_pct</t>
+          <t>FY2009</t>
         </is>
       </c>
       <c r="C189" t="n">
-        <v>460.73</v>
+        <v>24</v>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>percent total return, CNSWF USD, approximate, 10 years to 2026-05</t>
+          <t>percent</t>
         </is>
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>third_party</t>
+          <t>company</t>
         </is>
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>https://www.financecharts.com/stocks/CNSWF/performance/total-return-cagr</t>
-        </is>
-      </c>
-      <c r="G189" t="inlineStr"/>
+          <t>https://www.csisoftware.com/docs/default-source/investor-relations/presidents-letter/shareholder-letter---2009.pdf</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>2009 President's letter reported 24% ROIC for 2009.</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>aggregate_returns</t>
+          <t>roic_pct</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>total_return_15yr_pct</t>
+          <t>FY2010</t>
         </is>
       </c>
       <c r="C190" t="n">
-        <v>3597.83</v>
+        <v>25</v>
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>percent total return, CNSWF USD, approximate, 15 years to 2026-05</t>
+          <t>percent</t>
         </is>
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>third_party</t>
+          <t>company</t>
         </is>
       </c>
       <c r="F190" t="inlineStr">
         <is>
-          <t>https://www.financecharts.com/stocks/CNSWF/performance/total-return-cagr</t>
-        </is>
-      </c>
-      <c r="G190" t="inlineStr"/>
+          <t>https://www.csisoftware.com/docs/default-source/investor-relations/presidents-letter/shareholder-letter---2010.pdf</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>Reused from long-term-hold/holdings.json parent_long_run.</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>aggregate_returns</t>
+          <t>roic_plus_organic_pct</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>annualized_return_10yr_pct</t>
+          <t>FY2017</t>
         </is>
       </c>
       <c r="C191" t="n">
-        <v>19.63</v>
+        <v>33</v>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>percent per year, CSU.TO CAD, approximate, 10 years to 2026-09</t>
+          <t>percent, approximate</t>
         </is>
       </c>
       <c r="E191" t="inlineStr">
@@ -8123,45 +8221,247 @@
       </c>
       <c r="F191" t="inlineStr">
         <is>
-          <t>https://portfolioslab.com/symbol/CSU.TO</t>
+          <t>https://uploads-ssl.webflow.com/60e3655ca778911eb64b2a00/60f0777ead89beba9c51c0b3_Constellation-Software-Inc.-Shareholder-Letters.pdf</t>
         </is>
       </c>
       <c r="G191" t="inlineStr">
         <is>
-          <t>S&amp;P 500 averaged 13.95 percent over the same window per the same source.</t>
+          <t>ROIC+OGr 'remained relatively flat at 33%' in 2017 with shareholders' Average Invested Capital growing 29%. Corroborated by a second third-party source (bizalmanac.substack.com) citing the same 33% figure and 29% ROIC alone for FY2017.</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
+          <t>capex</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="C192" t="n">
+        <v>68</v>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>USD millions, approximate</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>third_party</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>https://www.stockopedia.com/share-prices/constellation-software-TSE:CSU/cashflow/</t>
+        </is>
+      </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>Aggregator-derived cash-flow-statement figure; not located in a company press release.</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>capex</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>FY2024</t>
+        </is>
+      </c>
+      <c r="C193" t="n">
+        <v>72</v>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>USD millions, approximate</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>third_party</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>https://www.stockopedia.com/share-prices/constellation-software-TSE:CSU/cashflow/</t>
+        </is>
+      </c>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>Aggregator-derived cash-flow-statement figure; not located in a company press release.</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>share_price_cad_year_end</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>IPO 2006-05-17</t>
+        </is>
+      </c>
+      <c r="C194" t="n">
+        <v>17</v>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>CAD, IPO offering price (not a fiscal year-end close)</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>third_party</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>https://www.cantechletter.com/2025/05/constellation-software-has-delivered-a-36000-return-since-its-ipo-is-it-still-a-buy/</t>
+        </is>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>Constellation listed on the TSX May 17, 2006 at an IPO price of C$17.00/share (first-day close C$18.30). Not independently confirmed from Constellation's own short-form prospectus (WebFetch unavailable); treated as third_party. No FY2006-FY2025 fiscal year-end closing price could be sourced via WebSearch in any of the five intake sweeps -- year end prices are gap for every one of the 19 fiscal years, per known issue 9.</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
           <t>aggregate_returns</t>
         </is>
       </c>
-      <c r="B192" t="inlineStr">
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>total_return_10yr_pct</t>
+        </is>
+      </c>
+      <c r="C195" t="n">
+        <v>460.73</v>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>percent total return, CNSWF USD, approximate, 10 years to 2026-05</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>third_party</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>https://www.financecharts.com/stocks/CNSWF/performance/total-return-cagr</t>
+        </is>
+      </c>
+      <c r="G195" t="inlineStr"/>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>aggregate_returns</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>total_return_15yr_pct</t>
+        </is>
+      </c>
+      <c r="C196" t="n">
+        <v>3597.83</v>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>percent total return, CNSWF USD, approximate, 15 years to 2026-05</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>third_party</t>
+        </is>
+      </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>https://www.financecharts.com/stocks/CNSWF/performance/total-return-cagr</t>
+        </is>
+      </c>
+      <c r="G196" t="inlineStr"/>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>aggregate_returns</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>annualized_return_10yr_pct</t>
+        </is>
+      </c>
+      <c r="C197" t="n">
+        <v>19.63</v>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>percent per year, CSU.TO CAD, approximate, 10 years to 2026-09</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>third_party</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>https://portfolioslab.com/symbol/CSU.TO</t>
+        </is>
+      </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>S&amp;P 500 averaged 13.95 percent over the same window per the same source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>aggregate_returns</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
         <is>
           <t>positive_years_count</t>
         </is>
       </c>
-      <c r="C192" t="n">
+      <c r="C198" t="n">
         <v>17</v>
       </c>
-      <c r="D192" t="inlineStr">
+      <c r="D198" t="inlineStr">
         <is>
           <t>positive calendar years out of since-listing total (2 negative), approximate</t>
         </is>
       </c>
-      <c r="E192" t="inlineStr">
+      <c r="E198" t="inlineStr">
         <is>
           <t>third_party</t>
         </is>
       </c>
-      <c r="F192" t="inlineStr">
+      <c r="F198" t="inlineStr">
         <is>
           <t>https://portfolioslab.com/symbol/CSU.TO</t>
         </is>
       </c>
-      <c r="G192" t="inlineStr"/>
+      <c r="G198" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8313,13 +8613,13 @@
         <v>2.2</v>
       </c>
       <c r="J3" t="n">
-        <v>116.73</v>
+        <v>96.62</v>
       </c>
       <c r="K3" t="n">
         <v>1099.9</v>
       </c>
       <c r="L3" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4">
@@ -8358,7 +8658,7 @@
         <v>2807</v>
       </c>
       <c r="L4" t="n">
-        <v>32</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5">
@@ -8375,12 +8675,18 @@
       <c r="C5" t="n">
         <v>20.63</v>
       </c>
+      <c r="D5" t="n">
+        <v>28.19</v>
+      </c>
       <c r="E5" t="n">
         <v>25.42</v>
       </c>
       <c r="F5" t="n">
         <v>20.63</v>
       </c>
+      <c r="G5" t="n">
+        <v>28.19</v>
+      </c>
       <c r="H5" t="n">
         <v>25.42</v>
       </c>
@@ -8388,7 +8694,7 @@
         <v>2.5</v>
       </c>
       <c r="J5" t="n">
-        <v>60.18</v>
+        <v>75.98</v>
       </c>
       <c r="K5" t="n">
         <v>5703</v>
@@ -8418,13 +8724,13 @@
         <v>0.76</v>
       </c>
       <c r="J6" t="n">
-        <v>83.7</v>
+        <v>83.05</v>
       </c>
       <c r="K6" t="n">
         <v>9703.9</v>
       </c>
       <c r="L6" t="n">
-        <v>64</v>
+        <v>80</v>
       </c>
     </row>
   </sheetData>
@@ -9142,14 +9448,14 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C11" t="n">
         <v>6</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>revenue, net_income_attributable, acquisitions_cash_spent, organic_growth_pct, cash_metric (adjusted_net_income)</t>
+          <t>revenue, net_income_attributable, cash_from_operations, acquisitions_cash_spent, organic_growth_pct, cash_metric (adjusted_net_income)</t>
         </is>
       </c>
     </row>
@@ -9250,14 +9556,14 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C17" t="n">
         <v>6</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>revenue, net_income_attributable, acquisitions_cash_spent, organic_growth_pct, cash_metric (fcfa2s)</t>
+          <t>revenue, net_income_attributable, cash_from_operations, acquisitions_cash_spent, organic_growth_pct, cash_metric (fcfa2s)</t>
         </is>
       </c>
     </row>

</xml_diff>